<commit_message>
Área 3: cierre #11 — revisión ERC + Rev B + kit de layout WN-SITE-CORE
</commit_message>
<xml_diff>
--- a/docs/hardware/wanomi_BOM_WN-SITE-CORE.xlsx
+++ b/docs/hardware/wanomi_BOM_WN-SITE-CORE.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="169">
-  <si>
-    <t xml:space="preserve">wanomi — BOM  ·  WN-SITE-CORE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Núcleo de sitio telco — monitoreo (Modo Connect + Sense)  ·  MCU ESP32-S3  ·  Alimentación -48 VDC planta  ·  feature/telco-support  ·  Sesión #10 — 2026-05-23</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="322" uniqueCount="192">
+  <si>
+    <t xml:space="preserve">wanomi — BOM  ·  WN-SITE-CORE (Rev B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Núcleo de sitio telco — monitoreo (Modo Connect + Sense)  ·  MCU ESP32-S3  ·  Alimentación -48 VDC planta  ·  feature/telco-support  ·  Rev B — Sesión #11 — 2026-05-24</t>
   </si>
   <si>
     <t xml:space="preserve">Ref</t>
@@ -101,7 +101,7 @@
     <t xml:space="preserve">Cátodo común</t>
   </si>
   <si>
-    <t xml:space="preserve">Verde OK / ámbar adv / rojo crítico</t>
+    <t xml:space="preserve">Verde OK / ámbar adv / rojo crítico · Rev B H-5: vía buffer 74AHCT1G125 (Ref 48)</t>
   </si>
   <si>
     <t xml:space="preserve">Alimentación</t>
@@ -116,7 +116,7 @@
     <t xml:space="preserve">Mouser</t>
   </si>
   <si>
-    <t xml:space="preserve">Primario -48V planta; 12/24V por DNP</t>
+    <t xml:space="preserve">Primario −48V planta. Rev B H-2: verificar rating transitorio de entrada (clamp 64A ~103V vs 75V).</t>
   </si>
   <si>
     <t xml:space="preserve">Buck 5V→3V3</t>
@@ -143,13 +143,13 @@
     <t xml:space="preserve">Fusible 1A + portafusible</t>
   </si>
   <si>
-    <t xml:space="preserve">TVS SMBJ58A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Clamp ~93V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Protección entrada DC</t>
+    <t xml:space="preserve">TVS entrada −48 V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMBJ64A (stand-off 64 V, clamp ~103 V)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-2: 58A→64A (cubre ecualización ~57-58V); coordinar clamp vs máx DC-DC</t>
   </si>
   <si>
     <t xml:space="preserve">MOSFET P reverse-pol.</t>
@@ -272,7 +272,7 @@
     <t xml:space="preserve">R sense 150Ω 0.1% + protección</t>
   </si>
   <si>
-    <t xml:space="preserve">Para sonda combustible</t>
+    <t xml:space="preserve">Para sonda combustible. Rev B H-1: alimentado por +V_LOOP (boost 24V, Ref 46).</t>
   </si>
   <si>
     <t xml:space="preserve">Entradas dig.</t>
@@ -284,13 +284,16 @@
     <t xml:space="preserve">2× quad TLP281-4 (8 canales)</t>
   </si>
   <si>
-    <t xml:space="preserve">Puerta/PIR/red/humo/contactos genset</t>
+    <t xml:space="preserve">Puerta/PIR/humo/contactos genset; IN3 (presencia AC) por relé ext./Modbus (Rev B H-3)</t>
   </si>
   <si>
     <t xml:space="preserve">Red entrada + TVS</t>
   </si>
   <si>
-    <t xml:space="preserve">R serie + TVS por canal</t>
+    <t xml:space="preserve">R serie ~560Ω (≥6 mA LED) + TVS + diodo antiparalelo /canal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-3: 4k7→560Ω; wetting +5V; COM=GND lógico</t>
   </si>
   <si>
     <t xml:space="preserve">Salidas (reserv.)</t>
@@ -461,6 +464,51 @@
     <t xml:space="preserve">Opcional según sitio</t>
   </si>
   <si>
+    <t xml:space="preserve">Boost +5V→24V (V_LOOP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MT3608 + L + Schottky + divisor 24V + caps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-1: alimenta lazo 4-20mA combustible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDT a PE (rayo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tubo descarga gaseosa, común-modo a tierra de sitio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-2: etapa de energía, surge de torre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buffer nivel WS2812</t>
+  </si>
+  <si>
+    <t xml:space="preserve">74AHCT1G125 3V3→5V (o Schottky en VDD del LED)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-5: VIH del WS2812 a 5V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jumper terminación RS-485</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Solder-bridge para R3 120Ω (extremo vs derivación)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-7: bus-end seleccionable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relé presencia 230VAC (opcional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bobina 230VAC→contacto seco a IN3; preferible utility del ATS por Modbus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rev B H-3: saca 220V de la placa</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total CORE — poblado en placa (1ª instancia)</t>
   </si>
   <si>
@@ -528,6 +576,27 @@
   </si>
   <si>
     <t xml:space="preserve">Costos: referencia en USD, sourcing AR (MercadoLibre/AliExpress) + especialidad (Mouser) + PCB JLCPCB lote 50. Precios indicativos a validar con cotización del proveedor.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambios Rev B (sesión #11) — cierre previo a captura KiCad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-1 [BLOQUEANTE]: +boost +5V→24V (V_LOOP, Ref 46) para el lazo 4-20mA de combustible; con +5V el sender de 2 hilos no arrancaba.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-2 [BLOQUEANTE]: TVS de entrada 58A→64A (ecualización ~57-58V); +GDT a PE (Ref 47) para rayo; verificar rating transitorio del DC-DC (clamp 103V vs 75V).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-3 [BLOQUEANTE]: 8 entradas re-tipificadas: wetting +5V, R serie ~560Ω (≥6mA LED), diodo antiparalelo/canal, COM=GND. IN3 (presencia AC) fuera de la placa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-5: buffer 74AHCT1G125 (Ref 48) para DIN del WS2812 (VIH a 5V).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-7: R3 (terminación RS-485) con jumper/solder-bridge (Ref 49): extremo vs derivación.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">H-4 / H-6: notas a validar (tasa efectiva ADS1115 para RMS; ventana de hold-up del supercap). Sin cambio de placa.</t>
   </si>
 </sst>
 </file>
@@ -538,7 +607,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="\$#,##0.00"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -657,6 +726,13 @@
     <font>
       <sz val="9"/>
       <color rgb="FF777777"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -803,8 +879,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="71">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -824,7 +904,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -832,7 +912,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -840,7 +920,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -848,7 +928,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -856,7 +936,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -864,11 +944,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -876,7 +956,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -884,7 +964,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -892,7 +972,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -900,7 +980,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -908,7 +988,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -916,11 +996,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -928,7 +1008,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -936,7 +1016,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -944,7 +1024,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -952,11 +1032,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="11" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -964,7 +1044,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -972,7 +1052,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="12" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -980,7 +1060,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -988,7 +1068,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="13" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -996,7 +1076,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1004,11 +1084,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="14" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1016,51 +1096,43 @@
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="15" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="15" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1081,6 +1153,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1336,1605 +1416,1745 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:J56"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5" t="s">
+      <c r="E5" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="8" t="n">
         <v>4.5</v>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="8" t="n">
         <f aca="false">E5*G5</f>
         <v>4.5</v>
       </c>
-      <c r="I5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="6" t="s">
+      <c r="I5" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="5" t="s">
+      <c r="E6" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="7" t="n">
+      <c r="G6" s="8" t="n">
         <v>0.8</v>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="8" t="n">
         <f aca="false">E6*G6</f>
         <v>0.8</v>
       </c>
-      <c r="I6" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J6" s="6"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="I6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="7"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="F7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="7" t="n">
+      <c r="G7" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="8" t="n">
         <f aca="false">E7*G7</f>
         <v>0.1</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
+      <c r="I7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="7"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="E8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="5" t="s">
+      <c r="E8" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="G8" s="7" t="n">
+      <c r="G8" s="8" t="n">
         <v>0.15</v>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="8" t="n">
         <f aca="false">E8*G8</f>
         <v>0.15</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="6" t="s">
+      <c r="I8" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
+    <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="B9" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="E9" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="9" t="s">
+      <c r="E9" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H9" s="12" t="n">
         <f aca="false">E9*G9</f>
         <v>12</v>
       </c>
-      <c r="I9" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="10" t="s">
+      <c r="I9" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="9" t="s">
+      <c r="B10" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="9" t="s">
+      <c r="E10" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="12" t="n">
         <v>1.5</v>
       </c>
-      <c r="H10" s="11" t="n">
+      <c r="H10" s="12" t="n">
         <f aca="false">E10*G10</f>
         <v>1.5</v>
       </c>
-      <c r="I10" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J10" s="10" t="s">
+      <c r="I10" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" s="11" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="9" t="s">
+      <c r="B11" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E11" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="9" t="s">
+      <c r="E11" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="12" t="n">
         <f aca="false">E11*G11</f>
         <v>3</v>
       </c>
-      <c r="I11" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="10" t="s">
+      <c r="I11" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="11" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="10"/>
-      <c r="E12" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="9" t="s">
+      <c r="D12" s="11"/>
+      <c r="E12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="H12" s="11" t="n">
+      <c r="H12" s="12" t="n">
         <f aca="false">E12*G12</f>
         <v>0.4</v>
       </c>
-      <c r="I12" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J12" s="10"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
+      <c r="I12" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J12" s="11"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="9" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="9" t="s">
+      <c r="E13" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="12" t="n">
         <v>0.2</v>
       </c>
-      <c r="H13" s="11" t="n">
+      <c r="H13" s="12" t="n">
         <f aca="false">E13*G13</f>
         <v>0.2</v>
       </c>
-      <c r="I13" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J13" s="10" t="s">
+      <c r="I13" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="11" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="B14" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E14" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="9" t="s">
+      <c r="E14" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="H14" s="11" t="n">
+      <c r="H14" s="12" t="n">
         <f aca="false">E14*G14</f>
         <v>0.3</v>
       </c>
-      <c r="I14" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J14" s="10"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
+      <c r="I14" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J14" s="11"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="9" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="B15" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="9" t="s">
+      <c r="E15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="12" t="n">
         <v>1.2</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H15" s="12" t="n">
         <f aca="false">E15*G15</f>
         <v>1.2</v>
       </c>
-      <c r="I15" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="J15" s="10" t="s">
+      <c r="I15" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J15" s="11" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="n">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="D16" s="14" t="s">
+      <c r="D16" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F16" s="13" t="s">
+      <c r="E16" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="15" t="n">
+      <c r="G16" s="16" t="n">
         <v>4.5</v>
       </c>
-      <c r="H16" s="15" t="n">
+      <c r="H16" s="16" t="n">
         <f aca="false">E16*G16</f>
         <v>4.5</v>
       </c>
-      <c r="I16" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J16" s="14" t="s">
+      <c r="I16" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J16" s="15" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="n">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C17" s="13" t="s">
+      <c r="C17" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D17" s="14" t="s">
+      <c r="D17" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="E17" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="E17" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="G17" s="15" t="n">
+      <c r="G17" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="H17" s="15" t="n">
+      <c r="H17" s="16" t="n">
         <f aca="false">E17*G17</f>
         <v>0.6</v>
       </c>
-      <c r="I17" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J17" s="14" t="s">
+      <c r="I17" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J17" s="15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="12" t="n">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="13" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="D18" s="14" t="s">
+      <c r="D18" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="E18" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="13" t="s">
+      <c r="E18" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G18" s="16" t="n">
         <v>3.5</v>
       </c>
-      <c r="H18" s="15" t="n">
+      <c r="H18" s="16" t="n">
         <f aca="false">E18*G18</f>
         <v>3.5</v>
       </c>
-      <c r="I18" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J18" s="14" t="s">
+      <c r="I18" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J18" s="15" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="n">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="13" t="s">
+      <c r="B19" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C19" s="13" t="s">
+      <c r="C19" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="D19" s="14" t="s">
+      <c r="D19" s="15" t="s">
         <v>59</v>
       </c>
-      <c r="E19" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="13" t="s">
+      <c r="E19" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="G19" s="15" t="n">
+      <c r="G19" s="16" t="n">
         <v>1.8</v>
       </c>
-      <c r="H19" s="15" t="n">
+      <c r="H19" s="16" t="n">
         <f aca="false">E19*G19</f>
         <v>1.8</v>
       </c>
-      <c r="I19" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J19" s="14"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="12" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="13" t="s">
+      <c r="I19" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J19" s="15"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="13" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="13" t="s">
+      <c r="C20" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D20" s="14" t="s">
+      <c r="D20" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="E20" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="13" t="s">
+      <c r="E20" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="G20" s="15" t="n">
+      <c r="G20" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="H20" s="15" t="n">
+      <c r="H20" s="16" t="n">
         <f aca="false">E20*G20</f>
         <v>0.5</v>
       </c>
-      <c r="I20" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J20" s="14"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="n">
+      <c r="I20" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J20" s="15"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="13" t="s">
+      <c r="B21" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="13" t="s">
+      <c r="C21" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="D21" s="14" t="s">
+      <c r="D21" s="15" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F21" s="13" t="s">
+      <c r="E21" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="G21" s="15" t="n">
+      <c r="G21" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="H21" s="15" t="n">
+      <c r="H21" s="16" t="n">
         <f aca="false">E21*G21</f>
         <v>4</v>
       </c>
-      <c r="I21" s="16" t="s">
+      <c r="I21" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="J21" s="14" t="s">
+      <c r="J21" s="15" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="n">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B22" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="D22" s="14" t="s">
+      <c r="D22" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="E22" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="13" t="s">
+      <c r="E22" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="G22" s="15" t="n">
+      <c r="G22" s="16" t="n">
         <v>1.2</v>
       </c>
-      <c r="H22" s="15" t="n">
+      <c r="H22" s="16" t="n">
         <f aca="false">E22*G22</f>
         <v>1.2</v>
       </c>
-      <c r="I22" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="J22" s="14"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17" t="n">
+      <c r="I22" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="J22" s="15"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D23" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="E23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="18" t="s">
+      <c r="E23" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="G23" s="20" t="n">
+      <c r="G23" s="21" t="n">
         <v>2.2</v>
       </c>
-      <c r="H23" s="20" t="n">
+      <c r="H23" s="21" t="n">
         <f aca="false">E23*G23</f>
         <v>2.2</v>
       </c>
-      <c r="I23" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J23" s="19" t="s">
+      <c r="I23" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="J23" s="20" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="n">
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C24" s="18" t="s">
+      <c r="C24" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="D24" s="19" t="s">
+      <c r="D24" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="E24" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="18" t="s">
+      <c r="E24" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="20" t="n">
+      <c r="G24" s="21" t="n">
         <v>2.5</v>
       </c>
-      <c r="H24" s="20" t="n">
+      <c r="H24" s="21" t="n">
         <f aca="false">E24*G24</f>
         <v>2.5</v>
       </c>
-      <c r="I24" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J24" s="19" t="s">
+      <c r="I24" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="J24" s="20" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="17" t="n">
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="18" t="s">
+      <c r="B25" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C25" s="18" t="s">
+      <c r="C25" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="D25" s="19" t="s">
+      <c r="D25" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="E25" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="18" t="s">
+      <c r="E25" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="G25" s="20" t="n">
+      <c r="G25" s="21" t="n">
         <v>22</v>
       </c>
-      <c r="H25" s="20" t="n">
+      <c r="H25" s="21" t="n">
         <f aca="false">E25*G25</f>
         <v>22</v>
       </c>
-      <c r="I25" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J25" s="19" t="s">
+      <c r="I25" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="J25" s="20" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="n">
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="18" t="s">
+      <c r="B26" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C26" s="18" t="s">
+      <c r="C26" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D26" s="19" t="s">
+      <c r="D26" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E26" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="18" t="s">
+      <c r="E26" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="20" t="n">
+      <c r="G26" s="21" t="n">
         <v>0.6</v>
       </c>
-      <c r="H26" s="20" t="n">
+      <c r="H26" s="21" t="n">
         <f aca="false">E26*G26</f>
         <v>0.6</v>
       </c>
-      <c r="I26" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J26" s="19" t="s">
+      <c r="I26" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="J26" s="20" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="17" t="n">
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="18" t="s">
+      <c r="B27" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="D27" s="19" t="s">
+      <c r="D27" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E27" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F27" s="18" t="s">
+      <c r="E27" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G27" s="20" t="n">
+      <c r="G27" s="21" t="n">
         <v>0.5</v>
       </c>
-      <c r="H27" s="20" t="n">
+      <c r="H27" s="21" t="n">
         <f aca="false">E27*G27</f>
         <v>0.5</v>
       </c>
-      <c r="I27" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="J27" s="19" t="s">
+      <c r="I27" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="J27" s="20" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="21" t="n">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="n">
         <v>24</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="23" t="s">
         <v>85</v>
       </c>
-      <c r="D28" s="23" t="s">
+      <c r="D28" s="24" t="s">
         <v>86</v>
       </c>
-      <c r="E28" s="21" t="n">
+      <c r="E28" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="F28" s="22" t="s">
+      <c r="F28" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="G28" s="24" t="n">
+      <c r="G28" s="25" t="n">
         <v>0.9</v>
       </c>
-      <c r="H28" s="24" t="n">
+      <c r="H28" s="25" t="n">
         <f aca="false">E28*G28</f>
         <v>1.8</v>
       </c>
-      <c r="I28" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J28" s="23" t="s">
+      <c r="I28" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="J28" s="24" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="n">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="23" t="s">
         <v>84</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="D29" s="23" t="s">
+      <c r="D29" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="E29" s="21" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="22" t="s">
+      <c r="E29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="G29" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="24" t="n">
+      <c r="G29" s="25" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H29" s="25" t="n">
         <f aca="false">E29*G29</f>
-        <v>1</v>
-      </c>
-      <c r="I29" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="J29" s="23"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="25" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="I29" s="23" t="s">
+        <v>16</v>
+      </c>
+      <c r="J29" s="24" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="26" t="n">
         <v>26</v>
       </c>
-      <c r="B30" s="26" t="s">
-        <v>90</v>
-      </c>
-      <c r="C30" s="26" t="s">
+      <c r="B30" s="27" t="s">
         <v>91</v>
       </c>
-      <c r="D30" s="27" t="s">
+      <c r="C30" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="E30" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="26" t="s">
+      <c r="D30" s="28" t="s">
+        <v>93</v>
+      </c>
+      <c r="E30" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="G30" s="28" t="n">
+      <c r="G30" s="29" t="n">
         <v>3</v>
       </c>
-      <c r="H30" s="28" t="n">
+      <c r="H30" s="29" t="n">
         <f aca="false">E30*G30</f>
         <v>3</v>
       </c>
-      <c r="I30" s="29" t="s">
+      <c r="I30" s="30" t="s">
         <v>64</v>
       </c>
-      <c r="J30" s="27" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="30" t="n">
+      <c r="J30" s="28" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="31" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="31" t="s">
-        <v>94</v>
-      </c>
-      <c r="C31" s="31" t="s">
+      <c r="B31" s="32" t="s">
         <v>95</v>
       </c>
-      <c r="D31" s="32" t="s">
+      <c r="C31" s="32" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="31" t="s">
+      <c r="D31" s="33" t="s">
+        <v>97</v>
+      </c>
+      <c r="E31" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G31" s="33" t="n">
+      <c r="G31" s="34" t="n">
         <v>1.8</v>
       </c>
-      <c r="H31" s="33" t="n">
+      <c r="H31" s="34" t="n">
         <f aca="false">E31*G31</f>
         <v>1.8</v>
       </c>
-      <c r="I31" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="J31" s="32" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="30" t="n">
+      <c r="I31" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="33" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="31" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="31" t="s">
-        <v>94</v>
-      </c>
-      <c r="C32" s="31" t="s">
-        <v>98</v>
-      </c>
-      <c r="D32" s="32" t="s">
+      <c r="B32" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" s="32" t="s">
         <v>99</v>
       </c>
-      <c r="E32" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="F32" s="31" t="s">
+      <c r="D32" s="33" t="s">
+        <v>100</v>
+      </c>
+      <c r="E32" s="31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="G32" s="33" t="n">
+      <c r="G32" s="34" t="n">
         <v>0.4</v>
       </c>
-      <c r="H32" s="33" t="n">
+      <c r="H32" s="34" t="n">
         <f aca="false">E32*G32</f>
         <v>0.4</v>
       </c>
-      <c r="I32" s="31" t="s">
-        <v>16</v>
-      </c>
-      <c r="J32" s="32"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="34" t="n">
+      <c r="I32" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="J32" s="33"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="35" t="n">
         <v>29</v>
       </c>
-      <c r="B33" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C33" s="35" t="s">
+      <c r="B33" s="36" t="s">
         <v>101</v>
       </c>
-      <c r="D33" s="36" t="s">
+      <c r="C33" s="36" t="s">
         <v>102</v>
       </c>
-      <c r="E33" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F33" s="35" t="s">
+      <c r="D33" s="37" t="s">
+        <v>103</v>
+      </c>
+      <c r="E33" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G33" s="37" t="n">
+      <c r="G33" s="38" t="n">
         <v>0.5</v>
       </c>
-      <c r="H33" s="37" t="n">
+      <c r="H33" s="38" t="n">
         <f aca="false">E33*G33</f>
         <v>0.5</v>
       </c>
-      <c r="I33" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J33" s="36"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="34" t="n">
+      <c r="I33" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" s="37"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="35" t="n">
         <v>30</v>
       </c>
-      <c r="B34" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C34" s="35" t="s">
-        <v>103</v>
-      </c>
-      <c r="D34" s="36" t="s">
+      <c r="B34" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C34" s="36" t="s">
         <v>104</v>
       </c>
-      <c r="E34" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F34" s="35" t="s">
+      <c r="D34" s="37" t="s">
+        <v>105</v>
+      </c>
+      <c r="E34" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G34" s="37" t="n">
+      <c r="G34" s="38" t="n">
         <v>0.4</v>
       </c>
-      <c r="H34" s="37" t="n">
+      <c r="H34" s="38" t="n">
         <f aca="false">E34*G34</f>
         <v>0.4</v>
       </c>
-      <c r="I34" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J34" s="36"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="34" t="n">
+      <c r="I34" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J34" s="37"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="35" t="n">
         <v>31</v>
       </c>
-      <c r="B35" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C35" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="D35" s="36" t="s">
+      <c r="B35" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" s="36" t="s">
         <v>106</v>
       </c>
-      <c r="E35" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="35" t="s">
+      <c r="D35" s="37" t="s">
+        <v>107</v>
+      </c>
+      <c r="E35" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G35" s="37" t="n">
+      <c r="G35" s="38" t="n">
         <v>0.5</v>
       </c>
-      <c r="H35" s="37" t="n">
+      <c r="H35" s="38" t="n">
         <f aca="false">E35*G35</f>
         <v>0.5</v>
       </c>
-      <c r="I35" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J35" s="36"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="34" t="n">
+      <c r="I35" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J35" s="37"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="35" t="n">
         <v>32</v>
       </c>
-      <c r="B36" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C36" s="35" t="s">
-        <v>107</v>
-      </c>
-      <c r="D36" s="36" t="s">
+      <c r="B36" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C36" s="36" t="s">
         <v>108</v>
       </c>
-      <c r="E36" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F36" s="35" t="s">
+      <c r="D36" s="37" t="s">
+        <v>109</v>
+      </c>
+      <c r="E36" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="37" t="n">
+      <c r="G36" s="38" t="n">
         <v>0.4</v>
       </c>
-      <c r="H36" s="37" t="n">
+      <c r="H36" s="38" t="n">
         <f aca="false">E36*G36</f>
         <v>0.4</v>
       </c>
-      <c r="I36" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J36" s="36"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="34" t="n">
+      <c r="I36" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J36" s="37"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="35" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C37" s="35" t="s">
-        <v>109</v>
-      </c>
-      <c r="D37" s="36" t="s">
+      <c r="B37" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C37" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="E37" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="35" t="s">
+      <c r="D37" s="37" t="s">
+        <v>111</v>
+      </c>
+      <c r="E37" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G37" s="37" t="n">
-        <v>1</v>
-      </c>
-      <c r="H37" s="37" t="n">
+      <c r="G37" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H37" s="38" t="n">
         <f aca="false">E37*G37</f>
         <v>1</v>
       </c>
-      <c r="I37" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J37" s="36"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="34" t="n">
+      <c r="I37" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J37" s="37"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="35" t="n">
         <v>34</v>
       </c>
-      <c r="B38" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C38" s="35" t="s">
-        <v>105</v>
-      </c>
-      <c r="D38" s="36" t="s">
-        <v>111</v>
-      </c>
-      <c r="E38" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="35" t="s">
+      <c r="B38" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C38" s="36" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" s="37" t="s">
+        <v>112</v>
+      </c>
+      <c r="E38" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="G38" s="37" t="n">
+      <c r="G38" s="38" t="n">
         <v>0.5</v>
       </c>
-      <c r="H38" s="37" t="n">
+      <c r="H38" s="38" t="n">
         <f aca="false">E38*G38</f>
         <v>0.5</v>
       </c>
-      <c r="I38" s="38" t="s">
+      <c r="I38" s="39" t="s">
         <v>64</v>
       </c>
-      <c r="J38" s="36"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="34" t="n">
+      <c r="J38" s="37"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="35" t="n">
         <v>35</v>
       </c>
-      <c r="B39" s="35" t="s">
-        <v>100</v>
-      </c>
-      <c r="C39" s="35" t="s">
-        <v>112</v>
-      </c>
-      <c r="D39" s="36" t="s">
+      <c r="B39" s="36" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="36" t="s">
         <v>113</v>
       </c>
-      <c r="E39" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F39" s="35" t="s">
+      <c r="D39" s="37" t="s">
+        <v>114</v>
+      </c>
+      <c r="E39" s="35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="G39" s="37" t="n">
+      <c r="G39" s="38" t="n">
         <v>0.3</v>
       </c>
-      <c r="H39" s="37" t="n">
+      <c r="H39" s="38" t="n">
         <f aca="false">E39*G39</f>
         <v>0.3</v>
       </c>
-      <c r="I39" s="35" t="s">
-        <v>16</v>
-      </c>
-      <c r="J39" s="36"/>
-    </row>
-    <row r="40" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="39" t="n">
+      <c r="I39" s="36" t="s">
+        <v>16</v>
+      </c>
+      <c r="J39" s="37"/>
+    </row>
+    <row r="40" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="40" t="n">
         <v>36</v>
       </c>
-      <c r="B40" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="C40" s="40" t="s">
+      <c r="B40" s="41" t="s">
         <v>115</v>
       </c>
-      <c r="D40" s="41" t="s">
+      <c r="C40" s="41" t="s">
         <v>116</v>
       </c>
-      <c r="E40" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F40" s="40" t="s">
+      <c r="D40" s="42" t="s">
         <v>117</v>
       </c>
-      <c r="G40" s="42" t="n">
+      <c r="E40" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="41" t="s">
+        <v>118</v>
+      </c>
+      <c r="G40" s="43" t="n">
         <v>6</v>
       </c>
-      <c r="H40" s="42" t="n">
+      <c r="H40" s="43" t="n">
         <f aca="false">E40*G40</f>
         <v>6</v>
       </c>
-      <c r="I40" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="J40" s="41" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="39" t="n">
+      <c r="I40" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="J40" s="42" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="40" t="n">
         <v>37</v>
       </c>
-      <c r="B41" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="C41" s="40" t="s">
-        <v>119</v>
-      </c>
-      <c r="D41" s="41" t="s">
+      <c r="B41" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="C41" s="41" t="s">
         <v>120</v>
       </c>
-      <c r="E41" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F41" s="40" t="s">
+      <c r="D41" s="42" t="s">
+        <v>121</v>
+      </c>
+      <c r="E41" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="41" t="s">
         <v>20</v>
       </c>
-      <c r="G41" s="42" t="n">
+      <c r="G41" s="43" t="n">
         <v>5</v>
       </c>
-      <c r="H41" s="42" t="n">
+      <c r="H41" s="43" t="n">
         <f aca="false">E41*G41</f>
         <v>5</v>
       </c>
-      <c r="I41" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="J41" s="41" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="39" t="n">
+      <c r="I41" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="J41" s="42" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="40" t="n">
         <v>38</v>
       </c>
-      <c r="B42" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="C42" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="D42" s="41" t="s">
+      <c r="B42" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="C42" s="41" t="s">
         <v>123</v>
       </c>
-      <c r="E42" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F42" s="40" t="s">
+      <c r="D42" s="42" t="s">
+        <v>124</v>
+      </c>
+      <c r="E42" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="41" t="s">
         <v>23</v>
       </c>
-      <c r="G42" s="42" t="n">
+      <c r="G42" s="43" t="n">
         <v>0.5</v>
       </c>
-      <c r="H42" s="42" t="n">
+      <c r="H42" s="43" t="n">
         <f aca="false">E42*G42</f>
         <v>0.5</v>
       </c>
-      <c r="I42" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="J42" s="41"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="39" t="n">
+      <c r="I42" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="J42" s="42"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="40" t="n">
         <v>39</v>
       </c>
-      <c r="B43" s="40" t="s">
-        <v>114</v>
-      </c>
-      <c r="C43" s="40" t="s">
-        <v>124</v>
-      </c>
-      <c r="D43" s="41" t="s">
+      <c r="B43" s="41" t="s">
+        <v>115</v>
+      </c>
+      <c r="C43" s="41" t="s">
         <v>125</v>
       </c>
-      <c r="E43" s="39" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="40" t="s">
+      <c r="D43" s="42" t="s">
         <v>126</v>
       </c>
-      <c r="G43" s="42" t="n">
+      <c r="E43" s="40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="G43" s="43" t="n">
         <v>0.4</v>
       </c>
-      <c r="H43" s="42" t="n">
+      <c r="H43" s="43" t="n">
         <f aca="false">E43*G43</f>
         <v>0.4</v>
       </c>
-      <c r="I43" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="J43" s="41"/>
-    </row>
-    <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="43" t="n">
+      <c r="I43" s="41" t="s">
+        <v>16</v>
+      </c>
+      <c r="J43" s="42"/>
+    </row>
+    <row r="44" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="44" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="44" t="s">
-        <v>127</v>
-      </c>
-      <c r="C44" s="44" t="s">
+      <c r="B44" s="45" t="s">
         <v>128</v>
       </c>
-      <c r="D44" s="45" t="s">
+      <c r="C44" s="45" t="s">
         <v>129</v>
       </c>
-      <c r="E44" s="43" t="n">
-        <v>1</v>
-      </c>
-      <c r="F44" s="44" t="s">
+      <c r="D44" s="46" t="s">
+        <v>130</v>
+      </c>
+      <c r="E44" s="44" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="45" t="s">
         <v>23</v>
       </c>
-      <c r="G44" s="46" t="n">
+      <c r="G44" s="47" t="n">
         <v>2.5</v>
       </c>
-      <c r="H44" s="46" t="n">
+      <c r="H44" s="47" t="n">
         <f aca="false">E44*G44</f>
         <v>2.5</v>
       </c>
-      <c r="I44" s="44" t="s">
-        <v>16</v>
-      </c>
-      <c r="J44" s="45"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="47" t="n">
+      <c r="I44" s="45" t="s">
+        <v>16</v>
+      </c>
+      <c r="J44" s="46"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="48" t="n">
         <v>41</v>
       </c>
-      <c r="B45" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C45" s="48" t="s">
+      <c r="B45" s="49" t="s">
         <v>131</v>
       </c>
-      <c r="D45" s="49" t="s">
+      <c r="C45" s="49" t="s">
         <v>132</v>
       </c>
-      <c r="E45" s="47" t="n">
+      <c r="D45" s="50" t="s">
+        <v>133</v>
+      </c>
+      <c r="E45" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="F45" s="48" t="s">
+      <c r="F45" s="49" t="s">
         <v>34</v>
       </c>
-      <c r="G45" s="50" t="n">
+      <c r="G45" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H45" s="50" t="n">
+      <c r="H45" s="51" t="n">
         <f aca="false">E45*G45</f>
         <v>6</v>
       </c>
-      <c r="I45" s="51" t="s">
-        <v>130</v>
-      </c>
-      <c r="J45" s="49" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="47" t="n">
+      <c r="I45" s="52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J45" s="50" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="48" t="n">
         <v>42</v>
       </c>
-      <c r="B46" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C46" s="48" t="s">
-        <v>134</v>
-      </c>
-      <c r="D46" s="49" t="s">
+      <c r="B46" s="49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C46" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="E46" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F46" s="48" t="s">
+      <c r="D46" s="50" t="s">
         <v>136</v>
       </c>
-      <c r="G46" s="50" t="n">
+      <c r="E46" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="49" t="s">
+        <v>137</v>
+      </c>
+      <c r="G46" s="51" t="n">
         <v>35</v>
       </c>
-      <c r="H46" s="50" t="n">
+      <c r="H46" s="51" t="n">
         <f aca="false">E46*G46</f>
         <v>35</v>
       </c>
-      <c r="I46" s="51" t="s">
-        <v>130</v>
-      </c>
-      <c r="J46" s="49" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="47" t="n">
+      <c r="I46" s="52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J46" s="50" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="48" t="n">
         <v>43</v>
       </c>
-      <c r="B47" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C47" s="48" t="s">
-        <v>138</v>
-      </c>
-      <c r="D47" s="49" t="s">
+      <c r="B47" s="49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C47" s="49" t="s">
         <v>139</v>
       </c>
-      <c r="E47" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F47" s="48" t="s">
+      <c r="D47" s="50" t="s">
+        <v>140</v>
+      </c>
+      <c r="E47" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="G47" s="50" t="n">
-        <v>1</v>
-      </c>
-      <c r="H47" s="50" t="n">
+      <c r="G47" s="51" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="51" t="n">
         <f aca="false">E47*G47</f>
         <v>1</v>
       </c>
-      <c r="I47" s="51" t="s">
-        <v>130</v>
-      </c>
-      <c r="J47" s="49" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="47" t="n">
+      <c r="I47" s="52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J47" s="50" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="48" t="n">
         <v>44</v>
       </c>
-      <c r="B48" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C48" s="48" t="s">
-        <v>141</v>
-      </c>
-      <c r="D48" s="49" t="s">
+      <c r="B48" s="49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C48" s="49" t="s">
         <v>142</v>
       </c>
-      <c r="E48" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="48" t="s">
+      <c r="D48" s="50" t="s">
+        <v>143</v>
+      </c>
+      <c r="E48" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="G48" s="50" t="n">
+      <c r="G48" s="51" t="n">
         <v>3</v>
       </c>
-      <c r="H48" s="50" t="n">
+      <c r="H48" s="51" t="n">
         <f aca="false">E48*G48</f>
         <v>3</v>
       </c>
-      <c r="I48" s="51" t="s">
-        <v>130</v>
-      </c>
-      <c r="J48" s="49"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="47" t="n">
+      <c r="I48" s="52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J48" s="50"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="48" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="48" t="s">
-        <v>130</v>
-      </c>
-      <c r="C49" s="48" t="s">
-        <v>143</v>
-      </c>
-      <c r="D49" s="49" t="s">
+      <c r="B49" s="49" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="49" t="s">
         <v>144</v>
       </c>
-      <c r="E49" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="48" t="s">
+      <c r="D49" s="50" t="s">
+        <v>145</v>
+      </c>
+      <c r="E49" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="G49" s="50" t="n">
+      <c r="G49" s="51" t="n">
         <v>8</v>
       </c>
-      <c r="H49" s="50" t="n">
+      <c r="H49" s="51" t="n">
         <f aca="false">E49*G49</f>
         <v>8</v>
       </c>
-      <c r="I49" s="51" t="s">
-        <v>130</v>
-      </c>
-      <c r="J49" s="49" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="52" t="s">
+      <c r="I49" s="52" t="s">
+        <v>131</v>
+      </c>
+      <c r="J49" s="50" t="s">
         <v>146</v>
       </c>
-      <c r="B51" s="52"/>
-      <c r="C51" s="52"/>
-      <c r="D51" s="52"/>
-      <c r="E51" s="52"/>
-      <c r="F51" s="52"/>
-      <c r="G51" s="52"/>
-      <c r="H51" s="53" t="n">
-        <f aca="false">SUMIF($I$5:$I$49,"Placa",$H$5:$H$49)</f>
-        <v>86.55</v>
-      </c>
-      <c r="I51" s="54"/>
-      <c r="J51" s="54"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="55" t="s">
+    </row>
+    <row r="50" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="9" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C50" s="10" t="s">
         <v>147</v>
       </c>
-      <c r="B52" s="55"/>
-      <c r="C52" s="55"/>
-      <c r="D52" s="55"/>
-      <c r="E52" s="55"/>
-      <c r="F52" s="55"/>
-      <c r="G52" s="55"/>
-      <c r="H52" s="56" t="n">
-        <f aca="false">SUMIF($I$5:$I$49,"Campo",$H$5:$H$49)</f>
-        <v>53</v>
-      </c>
-      <c r="I52" s="57"/>
-      <c r="J52" s="57"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="58" t="s">
+      <c r="D50" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="B53" s="58"/>
-      <c r="C53" s="58"/>
-      <c r="D53" s="58"/>
-      <c r="E53" s="58"/>
-      <c r="F53" s="58"/>
-      <c r="G53" s="58"/>
-      <c r="H53" s="59" t="n">
-        <f aca="false">SUMIF($I$5:$I$49,"DNP",$H$5:$H$49)</f>
+      <c r="E50" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="G50" s="12" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="H50" s="12" t="n">
+        <f aca="false">E50*G50</f>
+        <v>1.2</v>
+      </c>
+      <c r="I50" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J50" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="9" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="E51" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G51" s="9" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H51" s="12" t="n">
+        <f aca="false">E51*G51</f>
+        <v>0.5</v>
+      </c>
+      <c r="I51" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J51" s="11" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C52" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="E52" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G52" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H52" s="12" t="n">
+        <f aca="false">E52*G52</f>
+        <v>0.15</v>
+      </c>
+      <c r="I52" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J52" s="11" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="9" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C53" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="E53" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="G53" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H53" s="12" t="n">
+        <f aca="false">E53*G53</f>
+        <v>0.05</v>
+      </c>
+      <c r="I53" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="J53" s="11" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="9" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="C54" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="E54" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G54" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H54" s="12" t="n">
+        <f aca="false">E54*G54</f>
+        <v>3</v>
+      </c>
+      <c r="I54" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="J54" s="11" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="53" t="s">
+        <v>162</v>
+      </c>
+      <c r="B56" s="53"/>
+      <c r="C56" s="53"/>
+      <c r="D56" s="53"/>
+      <c r="E56" s="53"/>
+      <c r="F56" s="53"/>
+      <c r="G56" s="53"/>
+      <c r="H56" s="53" t="n">
+        <f aca="false">SUMIF($I$5:$I$54,"Placa",$H$5:$H$54)</f>
+        <v>88.75</v>
+      </c>
+      <c r="I56" s="53"/>
+      <c r="J56" s="53"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="54" t="s">
+        <v>163</v>
+      </c>
+      <c r="H57" s="55" t="n">
+        <f aca="false">SUMIF($I$5:$I$54,"Campo",$H$5:$H$54)</f>
+        <v>56</v>
+      </c>
+      <c r="I57" s="56"/>
+      <c r="J57" s="56"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="57" t="s">
+        <v>164</v>
+      </c>
+      <c r="H58" s="58" t="n">
+        <f aca="false">SUMIF($I$5:$I$54,"DNP",$H$5:$H$54)</f>
         <v>7.5</v>
       </c>
-      <c r="I53" s="60"/>
-      <c r="J53" s="60"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="61" t="s">
-        <v>149</v>
-      </c>
-      <c r="B54" s="61"/>
-      <c r="C54" s="61"/>
-      <c r="D54" s="61"/>
-      <c r="E54" s="61"/>
-      <c r="F54" s="61"/>
-      <c r="G54" s="61"/>
-      <c r="H54" s="62" t="n">
-        <f aca="false">SUMIF($I$5:$I$49,"Placa",$H$5:$H$49)+SUMIF($I$5:$I$49,"Campo",$H$5:$H$49)</f>
-        <v>139.55</v>
-      </c>
-      <c r="I54" s="63"/>
-      <c r="J54" s="63"/>
-    </row>
-    <row r="56" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="64" t="s">
-        <v>150</v>
-      </c>
-      <c r="B56" s="64"/>
-      <c r="C56" s="64"/>
-      <c r="D56" s="64"/>
-      <c r="E56" s="64"/>
-      <c r="F56" s="64"/>
-      <c r="G56" s="64"/>
-      <c r="H56" s="64"/>
-      <c r="I56" s="64"/>
-      <c r="J56" s="64"/>
+      <c r="I58" s="59"/>
+      <c r="J58" s="59"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="60" t="s">
+        <v>165</v>
+      </c>
+      <c r="H59" s="61" t="n">
+        <f aca="false">SUMIF($I$5:$I$54,"Placa",$H$5:$H$54)+SUMIF($I$5:$I$54,"Campo",$H$5:$H$54)</f>
+        <v>144.75</v>
+      </c>
+      <c r="I59" s="62"/>
+      <c r="J59" s="62"/>
+    </row>
+    <row r="61" customFormat="false" ht="450" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="63" t="s">
+        <v>166</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -2961,112 +3181,147 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="100"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="100"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="65" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="66"/>
+      <c r="A1" s="64" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="65"/>
     </row>
     <row r="3" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="67" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="66" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="66" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="66" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="66" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="66" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="66" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="66"/>
+      <c r="A3" s="66" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="65" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="65" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="65" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="65" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="65" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="65" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="65"/>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="67" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="66" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="66" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="66" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="66"/>
+      <c r="A11" s="66" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="65" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="65" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="65" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="65"/>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="68" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="66" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="66" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="66" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="66" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="66"/>
-    </row>
-    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="69" t="s">
-        <v>168</v>
+      <c r="A16" s="67" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="65" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="65" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="65" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="65" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="65"/>
+    </row>
+    <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="68" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="69" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="70" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="70" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="70" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="70" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="70" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="70" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>